<commit_message>
Added engineering fee, board price, and PCBA service to the BOM.. Updated BOM and README (now Readme also have running total)
</commit_message>
<xml_diff>
--- a/BOM/all.xlsx
+++ b/BOM/all.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="157">
   <si>
     <t>Number</t>
   </si>
@@ -264,6 +264,21 @@
     <t>https://tk.tokopedia.com/ZSxcP4PVw/</t>
   </si>
   <si>
+    <t>Engineering Fee</t>
+  </si>
+  <si>
+    <t>https://jlcpcb.com/</t>
+  </si>
+  <si>
+    <t>PCB Board</t>
+  </si>
+  <si>
+    <t>PCBA Price</t>
+  </si>
+  <si>
+    <t>If enabled PCBA option</t>
+  </si>
+  <si>
     <t>TPOWER TP4056</t>
   </si>
   <si>
@@ -456,7 +471,7 @@
     <t>https://tk.tokopedia.com/ZSxcDnUcT/</t>
   </si>
   <si>
-    <t>https://tk.tokopedia.com/ZSxcUYBUF/</t>
+    <t>https://tk.tokopedia.com/ZSxc5xuDv/</t>
   </si>
   <si>
     <t>Price</t>
@@ -475,7 +490,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -529,6 +544,12 @@
       <name val="Poppins"/>
     </font>
     <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Open Sauce One&quot;"/>
+    </font>
+    <font>
       <b/>
       <color theme="1"/>
       <name val="Poppins"/>
@@ -554,7 +575,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -603,16 +624,10 @@
     <xf borderId="0" fillId="2" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -622,13 +637,16 @@
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" wrapText="0"/>
+      <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -937,7 +955,7 @@
         <v>13</v>
       </c>
       <c r="H3" s="8">
-        <f t="shared" ref="H3:H26" si="1">H2+F3</f>
+        <f t="shared" ref="H3:H29" si="1">H2+F3</f>
         <v>4.4734</v>
       </c>
       <c r="I3" s="9"/>
@@ -1486,7 +1504,7 @@
         <v>9.0E-4</v>
       </c>
       <c r="F23" s="7">
-        <f t="shared" ref="F23:F26" si="4">D23*E23</f>
+        <f t="shared" ref="F23:F29" si="4">D23*E23</f>
         <v>0.0027</v>
       </c>
       <c r="G23" s="6" t="s">
@@ -1582,1021 +1600,178 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="7"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="16"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="16"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="16"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="16"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="16"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="16"/>
-      <c r="B36" s="16"/>
-      <c r="C36" s="16"/>
-      <c r="D36" s="16"/>
-      <c r="E36" s="16"/>
-      <c r="F36" s="16"/>
-      <c r="G36" s="16"/>
-      <c r="H36" s="16"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="16"/>
-      <c r="B37" s="16"/>
-      <c r="C37" s="16"/>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16"/>
-      <c r="F37" s="16"/>
-      <c r="G37" s="16"/>
-      <c r="H37" s="16"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="16"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="16"/>
-      <c r="D38" s="16"/>
-      <c r="E38" s="16"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="16"/>
-      <c r="H38" s="16"/>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="G2"/>
-    <hyperlink r:id="rId2" ref="G3"/>
-    <hyperlink r:id="rId3" ref="G4"/>
-    <hyperlink r:id="rId4" ref="G5"/>
-    <hyperlink r:id="rId5" ref="G6"/>
-    <hyperlink r:id="rId6" ref="G7"/>
-    <hyperlink r:id="rId7" ref="G8"/>
-    <hyperlink r:id="rId8" ref="G9"/>
-    <hyperlink r:id="rId9" ref="G10"/>
-    <hyperlink r:id="rId10" ref="G11"/>
-    <hyperlink r:id="rId11" ref="G12"/>
-    <hyperlink r:id="rId12" ref="G13"/>
-    <hyperlink r:id="rId13" ref="G14"/>
-    <hyperlink r:id="rId14" ref="G15"/>
-    <hyperlink r:id="rId15" ref="G16"/>
-    <hyperlink r:id="rId16" ref="G17"/>
-    <hyperlink r:id="rId17" ref="G18"/>
-    <hyperlink r:id="rId18" ref="G19"/>
-    <hyperlink r:id="rId19" ref="G20"/>
-    <hyperlink r:id="rId20" ref="G21"/>
-    <hyperlink r:id="rId21" ref="G22"/>
-    <hyperlink r:id="rId22" ref="G23"/>
-    <hyperlink r:id="rId23" ref="G24"/>
-    <hyperlink r:id="rId24" ref="G25"/>
-    <hyperlink r:id="rId25" ref="G26"/>
-  </hyperlinks>
-  <drawing r:id="rId26"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="2" max="2" width="27.88"/>
-    <col customWidth="1" min="3" max="3" width="21.13"/>
-    <col customWidth="1" min="8" max="8" width="24.25"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3">
-        <v>1.0</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D2" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E2" s="21">
-        <v>0.1194</v>
-      </c>
-      <c r="F2" s="21">
-        <v>0.1194</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="H2" s="8">
-        <f>F2</f>
-        <v>0.1194</v>
-      </c>
-      <c r="I2" s="16"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3">
-        <v>2.0</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D3" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E3" s="5">
-        <v>0.0428</v>
-      </c>
-      <c r="F3" s="5">
-        <v>0.0428</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H3" s="8">
-        <f t="shared" ref="H3:H10" si="1">H2+F3</f>
-        <v>0.1622</v>
-      </c>
-      <c r="I3" s="16"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3">
-        <v>3.0</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D4" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E4" s="5">
-        <v>0.0786</v>
-      </c>
-      <c r="F4" s="5">
-        <v>0.0786</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="H4" s="8">
-        <f t="shared" si="1"/>
-        <v>0.2408</v>
-      </c>
-      <c r="I4" s="16"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3">
-        <v>4.0</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="5">
-        <v>0.0575</v>
-      </c>
-      <c r="F5" s="5">
-        <v>0.0575</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="H5" s="8">
-        <f t="shared" si="1"/>
-        <v>0.2983</v>
-      </c>
-      <c r="I5" s="16"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D6" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E6" s="5">
-        <v>0.0742</v>
-      </c>
-      <c r="F6" s="7">
-        <f>D6*E6</f>
-        <v>0.1484</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="H6" s="8">
-        <f t="shared" si="1"/>
-        <v>0.4467</v>
-      </c>
-      <c r="I6" s="16"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3">
-        <v>6.0</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D7" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0.007</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0.007</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="H7" s="8">
-        <f t="shared" si="1"/>
-        <v>0.4537</v>
-      </c>
-      <c r="I7" s="16"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3">
-        <v>7.0</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="D8" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E8" s="5">
-        <v>0.0163</v>
-      </c>
-      <c r="F8" s="5">
-        <v>0.0163</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="H8" s="8">
-        <f t="shared" si="1"/>
-        <v>0.47</v>
-      </c>
-      <c r="I8" s="16"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3">
-        <v>8.0</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D9" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0.0381</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0.0381</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="H9" s="8">
-        <f t="shared" si="1"/>
-        <v>0.5081</v>
-      </c>
-      <c r="I9" s="16"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D10" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0.2076</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0.2076</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="H10" s="8">
-        <f t="shared" si="1"/>
-        <v>0.7157</v>
-      </c>
-      <c r="I10" s="16"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="D11" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0.204</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0.204</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="H11" s="8">
-        <f>H10+E11</f>
-        <v>0.9197</v>
-      </c>
-      <c r="I11" s="16"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3">
-        <v>11.0</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="D12" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E12" s="5">
-        <v>4.83</v>
-      </c>
-      <c r="F12" s="5">
-        <v>4.83</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="H12" s="8">
-        <f t="shared" ref="H12:H27" si="2">H11+F12</f>
-        <v>5.7497</v>
-      </c>
-      <c r="I12" s="16"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3">
-        <v>12.0</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="D13" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E13" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F13" s="7">
-        <f t="shared" ref="F13:F27" si="3">D13*E13</f>
-        <v>0.0006</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H13" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7503</v>
-      </c>
-      <c r="I13" s="16"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3">
-        <v>13.0</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D14" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E14" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F14" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0006</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="H14" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7509</v>
-      </c>
-      <c r="I14" s="16"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3">
-        <v>14.0</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D15" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E15" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F15" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0003</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="H15" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7512</v>
-      </c>
-      <c r="I15" s="16"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3">
-        <v>15.0</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E16" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F16" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0003</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="H16" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7515</v>
-      </c>
-      <c r="I16" s="16"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3">
-        <v>16.0</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E17" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F17" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0006</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7521</v>
-      </c>
-      <c r="I17" s="16"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3">
-        <v>17.0</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D18" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E18" s="5">
-        <v>2.0E-4</v>
-      </c>
-      <c r="F18" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0002</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H18" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7523</v>
-      </c>
-      <c r="I18" s="16"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3">
-        <v>18.0</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D19" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E19" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F19" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0003</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="H19" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7526</v>
-      </c>
-      <c r="I19" s="16"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3">
-        <v>19.0</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D20" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E20" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F20" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0006</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="H20" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7532</v>
-      </c>
-      <c r="I20" s="16"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3">
-        <v>20.0</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D21" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E21" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F21" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0003</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="H21" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7535</v>
-      </c>
-      <c r="I21" s="16"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3">
-        <v>21.0</v>
-      </c>
-      <c r="B22" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="D22" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E22" s="5">
-        <v>0.0019</v>
-      </c>
-      <c r="F22" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0038</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7573</v>
-      </c>
-      <c r="I22" s="16"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="3">
-        <v>22.0</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D23" s="5">
-        <v>2.0</v>
-      </c>
-      <c r="E23" s="5">
-        <v>0.0027</v>
-      </c>
-      <c r="F23" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0054</v>
-      </c>
-      <c r="G23" s="22" t="s">
-        <v>141</v>
-      </c>
-      <c r="H23" s="8">
-        <f t="shared" si="2"/>
-        <v>5.7627</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3">
-        <v>23.0</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D24" s="5">
-        <v>1.0</v>
-      </c>
-      <c r="E24" s="5">
-        <v>3.0E-4</v>
-      </c>
-      <c r="F24" s="7">
-        <f t="shared" si="3"/>
-        <v>0.0003</v>
-      </c>
-      <c r="G24" s="22" t="s">
-        <v>143</v>
-      </c>
-      <c r="H24" s="8">
-        <f t="shared" si="2"/>
-        <v>5.763</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3">
-        <v>24.0</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D25" s="4">
-        <v>6.0</v>
-      </c>
-      <c r="E25" s="4">
-        <v>0.001</v>
-      </c>
-      <c r="F25" s="13">
-        <f t="shared" si="3"/>
-        <v>0.006</v>
-      </c>
-      <c r="G25" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="H25" s="3">
-        <f t="shared" si="2"/>
-        <v>5.769</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="3">
-        <v>25.0</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="D26" s="4">
-        <v>4.0</v>
-      </c>
-      <c r="E26" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="F26" s="13">
-        <f t="shared" si="3"/>
-        <v>0.2</v>
-      </c>
-      <c r="G26" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="H26" s="8">
-        <f t="shared" si="2"/>
-        <v>5.969</v>
-      </c>
-    </row>
-    <row r="27">
       <c r="A27" s="3">
         <v>26.0</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>81</v>
+      <c r="B27" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>83</v>
       </c>
       <c r="D27" s="5">
-        <v>4.0</v>
+        <v>1.0</v>
       </c>
       <c r="E27" s="5">
-        <v>0.054</v>
+        <v>24.0</v>
       </c>
       <c r="F27" s="7">
-        <f t="shared" si="3"/>
-        <v>0.216</v>
-      </c>
-      <c r="G27" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="H27" s="8">
-        <f t="shared" si="2"/>
-        <v>6.185</v>
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" s="7">
+        <f t="shared" si="1"/>
+        <v>36.2785</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="24"/>
+      <c r="A28" s="3">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="11">
+        <v>1.6</v>
+      </c>
+      <c r="F28" s="17">
+        <f t="shared" si="4"/>
+        <v>1.6</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="17">
+        <f t="shared" si="1"/>
+        <v>37.8785</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="10"/>
+      <c r="A29" s="3">
+        <v>28.0</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="11">
+        <v>1.0</v>
+      </c>
+      <c r="E29" s="11">
+        <v>42.17</v>
+      </c>
+      <c r="F29" s="17">
+        <f t="shared" si="4"/>
+        <v>42.17</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" s="17">
+        <f t="shared" si="1"/>
+        <v>80.0485</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
+      <c r="A30" s="3"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
     </row>
     <row r="31">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
+      <c r="A31" s="3"/>
+      <c r="B31" s="17"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
     </row>
     <row r="32">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
+      <c r="A32" s="17"/>
+      <c r="B32" s="17"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
     </row>
     <row r="33">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
+      <c r="A33" s="17"/>
+      <c r="B33" s="17"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
     </row>
     <row r="34">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
+      <c r="A34" s="17"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
     </row>
     <row r="35">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
+      <c r="A35" s="17"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
     </row>
     <row r="36">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="10"/>
+      <c r="A36" s="17"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="17"/>
+      <c r="E36" s="17"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="17"/>
+      <c r="H36" s="17"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="17"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="17"/>
+      <c r="B38" s="17"/>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+      <c r="H38" s="17"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2626,8 +1801,946 @@
     <hyperlink r:id="rId24" ref="G25"/>
     <hyperlink r:id="rId25" ref="G26"/>
     <hyperlink r:id="rId26" ref="G27"/>
+    <hyperlink r:id="rId27" ref="G28"/>
+    <hyperlink r:id="rId28" ref="G29"/>
   </hyperlinks>
-  <drawing r:id="rId27"/>
+  <drawing r:id="rId29"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="27.88"/>
+    <col customWidth="1" min="3" max="3" width="21.13"/>
+    <col customWidth="1" min="8" max="8" width="24.25"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E2" s="19">
+        <v>0.1194</v>
+      </c>
+      <c r="F2" s="19">
+        <v>0.1194</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" s="8">
+        <f>F2</f>
+        <v>0.1194</v>
+      </c>
+      <c r="I2" s="17"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.0428</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0.0428</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" s="8">
+        <f t="shared" ref="H3:H10" si="1">H2+F3</f>
+        <v>0.1622</v>
+      </c>
+      <c r="I3" s="17"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E4" s="5">
+        <v>0.0786</v>
+      </c>
+      <c r="F4" s="5">
+        <v>0.0786</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H4" s="8">
+        <f t="shared" si="1"/>
+        <v>0.2408</v>
+      </c>
+      <c r="I4" s="17"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="7"/>
+      <c r="E5" s="5">
+        <v>0.0575</v>
+      </c>
+      <c r="F5" s="5">
+        <v>0.0575</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="8">
+        <f t="shared" si="1"/>
+        <v>0.2983</v>
+      </c>
+      <c r="I5" s="17"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D6" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E6" s="5">
+        <v>0.0742</v>
+      </c>
+      <c r="F6" s="7">
+        <f>D6*E6</f>
+        <v>0.1484</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="H6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.4467</v>
+      </c>
+      <c r="I6" s="17"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D7" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E7" s="5">
+        <v>0.007</v>
+      </c>
+      <c r="F7" s="5">
+        <v>0.007</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="H7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.4537</v>
+      </c>
+      <c r="I7" s="17"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0.0163</v>
+      </c>
+      <c r="F8" s="5">
+        <v>0.0163</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="H8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.47</v>
+      </c>
+      <c r="I8" s="17"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="D9" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0.0381</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0.0381</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H9" s="8">
+        <f t="shared" si="1"/>
+        <v>0.5081</v>
+      </c>
+      <c r="I9" s="17"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.2076</v>
+      </c>
+      <c r="F10" s="5">
+        <v>0.2076</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H10" s="8">
+        <f t="shared" si="1"/>
+        <v>0.7157</v>
+      </c>
+      <c r="I10" s="17"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D11" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0.204</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0.204</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="H11" s="8">
+        <f>H10+E11</f>
+        <v>0.9197</v>
+      </c>
+      <c r="I11" s="17"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3">
+        <v>11.0</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D12" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>4.83</v>
+      </c>
+      <c r="F12" s="5">
+        <v>4.83</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="H12" s="8">
+        <f t="shared" ref="H12:H29" si="2">H11+F12</f>
+        <v>5.7497</v>
+      </c>
+      <c r="I12" s="17"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3">
+        <v>12.0</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D13" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E13" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F13" s="7">
+        <f t="shared" ref="F13:F29" si="3">D13*E13</f>
+        <v>0.0006</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="H13" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7503</v>
+      </c>
+      <c r="I13" s="17"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3">
+        <v>13.0</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F14" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0006</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="H14" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7509</v>
+      </c>
+      <c r="I14" s="17"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F15" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0003</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7512</v>
+      </c>
+      <c r="I15" s="17"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3">
+        <v>15.0</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F16" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0003</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7515</v>
+      </c>
+      <c r="I16" s="17"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3">
+        <v>16.0</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D17" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F17" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0006</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H17" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7521</v>
+      </c>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3">
+        <v>17.0</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D18" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2.0E-4</v>
+      </c>
+      <c r="F18" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0002</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="H18" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7523</v>
+      </c>
+      <c r="I18" s="17"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3">
+        <v>18.0</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D19" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F19" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0003</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H19" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7526</v>
+      </c>
+      <c r="I19" s="17"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D20" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F20" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0006</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="H20" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7532</v>
+      </c>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3">
+        <v>20.0</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D21" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E21" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F21" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0003</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="H21" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7535</v>
+      </c>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3">
+        <v>21.0</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="D22" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0.0019</v>
+      </c>
+      <c r="F22" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0038</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H22" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7573</v>
+      </c>
+      <c r="I22" s="17"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3">
+        <v>22.0</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D23" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0.0027</v>
+      </c>
+      <c r="F23" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0054</v>
+      </c>
+      <c r="G23" s="20" t="s">
+        <v>146</v>
+      </c>
+      <c r="H23" s="8">
+        <f t="shared" si="2"/>
+        <v>5.7627</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3">
+        <v>23.0</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D24" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>3.0E-4</v>
+      </c>
+      <c r="F24" s="7">
+        <f t="shared" si="3"/>
+        <v>0.0003</v>
+      </c>
+      <c r="G24" s="20" t="s">
+        <v>148</v>
+      </c>
+      <c r="H24" s="8">
+        <f t="shared" si="2"/>
+        <v>5.763</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3">
+        <v>24.0</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="D25" s="4">
+        <v>6.0</v>
+      </c>
+      <c r="E25" s="4">
+        <v>0.001</v>
+      </c>
+      <c r="F25" s="13">
+        <f t="shared" si="3"/>
+        <v>0.006</v>
+      </c>
+      <c r="G25" s="14" t="s">
+        <v>151</v>
+      </c>
+      <c r="H25" s="3">
+        <f t="shared" si="2"/>
+        <v>5.769</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3">
+        <v>25.0</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D26" s="4">
+        <v>4.0</v>
+      </c>
+      <c r="E26" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="F26" s="13">
+        <f t="shared" si="3"/>
+        <v>0.2</v>
+      </c>
+      <c r="G26" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="H26" s="8">
+        <f t="shared" si="2"/>
+        <v>5.969</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3">
+        <v>26.0</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D27" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0.054</v>
+      </c>
+      <c r="F27" s="7">
+        <f t="shared" si="3"/>
+        <v>0.216</v>
+      </c>
+      <c r="G27" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="H27" s="8">
+        <f t="shared" si="2"/>
+        <v>6.185</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="D28" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="E28" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="F28" s="10">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="23">
+        <f t="shared" si="2"/>
+        <v>7.185</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22">
+        <v>28.0</v>
+      </c>
+      <c r="B29" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C29" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="E29" s="22">
+        <v>70.25</v>
+      </c>
+      <c r="F29" s="10">
+        <f t="shared" si="3"/>
+        <v>70.25</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" s="10">
+        <f t="shared" si="2"/>
+        <v>77.435</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="10"/>
+      <c r="H30" s="10"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10"/>
+      <c r="B31" s="10"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="10"/>
+      <c r="H31" s="10"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10"/>
+      <c r="B32" s="10"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="10"/>
+      <c r="H32" s="10"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="10"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="10"/>
+      <c r="G34" s="10"/>
+      <c r="H34" s="10"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10"/>
+      <c r="B35" s="10"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="10"/>
+      <c r="G35" s="10"/>
+      <c r="H35" s="10"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="10"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="10"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="G2"/>
+    <hyperlink r:id="rId2" ref="G3"/>
+    <hyperlink r:id="rId3" ref="G4"/>
+    <hyperlink r:id="rId4" ref="G5"/>
+    <hyperlink r:id="rId5" ref="G6"/>
+    <hyperlink r:id="rId6" ref="G7"/>
+    <hyperlink r:id="rId7" ref="G8"/>
+    <hyperlink r:id="rId8" ref="G9"/>
+    <hyperlink r:id="rId9" ref="G10"/>
+    <hyperlink r:id="rId10" ref="G11"/>
+    <hyperlink r:id="rId11" ref="G12"/>
+    <hyperlink r:id="rId12" ref="G13"/>
+    <hyperlink r:id="rId13" ref="G14"/>
+    <hyperlink r:id="rId14" ref="G15"/>
+    <hyperlink r:id="rId15" ref="G16"/>
+    <hyperlink r:id="rId16" ref="G17"/>
+    <hyperlink r:id="rId17" ref="G18"/>
+    <hyperlink r:id="rId18" ref="G19"/>
+    <hyperlink r:id="rId19" ref="G20"/>
+    <hyperlink r:id="rId20" ref="G21"/>
+    <hyperlink r:id="rId21" ref="G22"/>
+    <hyperlink r:id="rId22" ref="G23"/>
+    <hyperlink r:id="rId23" ref="G24"/>
+    <hyperlink r:id="rId24" ref="G25"/>
+    <hyperlink r:id="rId25" ref="G26"/>
+    <hyperlink r:id="rId26" ref="G27"/>
+    <hyperlink r:id="rId27" ref="G28"/>
+    <hyperlink r:id="rId28" ref="G29"/>
+  </hyperlinks>
+  <drawing r:id="rId29"/>
 </worksheet>
 </file>
 
@@ -2639,41 +2752,41 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="25" t="s">
-        <v>148</v>
-      </c>
-      <c r="C1" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="D1" s="16"/>
+      <c r="B1" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" s="17"/>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3">
-        <v>12.2785</v>
+        <v>80.0485</v>
       </c>
       <c r="C2" s="11">
-        <v>12.2785</v>
-      </c>
-      <c r="D2" s="16"/>
+        <v>80.0485</v>
+      </c>
+      <c r="D2" s="17"/>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B3" s="3">
-        <v>6.185</v>
-      </c>
-      <c r="C3" s="16">
+        <v>77.435</v>
+      </c>
+      <c r="C3" s="17">
         <f>C2+B3</f>
-        <v>18.4635</v>
-      </c>
-      <c r="D3" s="16"/>
+        <v>157.4835</v>
+      </c>
+      <c r="D3" s="17"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>